<commit_message>
orders-deselected-waving changes: temp files
</commit_message>
<xml_diff>
--- a/orders-deselected-waving/WarehouseDetail_records(orders-deselected-waving).xlsx
+++ b/orders-deselected-waving/WarehouseDetail_records(orders-deselected-waving).xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/rndc/Desktop/Work related/Documents/orders-deselected-waving/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7EFDABCF-0DBC-7941-9816-068C33FCBE15}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5367E56D-E4B0-3C4D-9B7C-7EFFCF791FAF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="760" windowWidth="34560" windowHeight="20500" xr2:uid="{00000000-000D-0000-FFFF-FFFF01000000}"/>
+    <workbookView xWindow="34560" yWindow="0" windowWidth="19200" windowHeight="21600" xr2:uid="{00000000-000D-0000-FFFF-FFFF01000000}"/>
   </bookViews>
   <sheets>
     <sheet name="(main group)" sheetId="6" r:id="rId1"/>
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="754" uniqueCount="181">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="754" uniqueCount="185">
   <si>
     <t>Current</t>
   </si>
@@ -1505,9 +1505,6 @@
     <t>Excluded:</t>
   </si>
   <si>
-    <t>Null</t>
-  </si>
-  <si>
     <t>-</t>
   </si>
   <si>
@@ -1518,6 +1515,21 @@
   </si>
   <si>
     <t>{"alertName":"STANDARD ORDERS DESELECTED DURING WAVING","dataSource":"MAWM","database":{"connection":"MAPRD_NEW","type":"MySQL","uri":"jdbc:{host}:{port}/information_schema"},"email":{"subject":"Splunk Alert: $alertName$","body":"&lt;pre&gt;The alert condition for ''$name$'' was triggered.&lt;/pre&gt;","fromEmail":"wms-tools-noreply@rndc-usa.com","toEmail":"Teppi.Waxman@RNDC-USA.COM, stanley.monis@rndc-usa.com, SeoFoo.Dang@RNDC-USA.COM, Vincent.Labasan@RNDC-USA.COM, Amorsolo.Angco@rndc-usa.com, Wallace.Moniz@RNDC-USA.COM, Reoben.Aquino@RNDC-USA.COM, ashlyn.javier@rndc-usa.com CC: wmsinternal@rndc-usa.com, wmsconsultant@rndc-usa.com, WMSMSPSupport@RNDC-USA.COM","footer":"","attachment":["link-to-alert","link-to-results","inline-table"]},"sql":"SELECT DE.org_id, DE.order_id, O.ext_route_id, DE.order_planning_run_id, DE.deselected_orders, DE.deselected_order_lines, DE.updated_by, DE.created_timestamp FROM   default_dcorder.dco_plan_run_deselect_count DE join default_dcorder.dco_order_plan_run_strategy PLA ON DE.order_planning_run_id = PLA.order_planning_run_id AND PLA.org_id = DE.org_id left join default_dcorder.dco_order O ON O.order_id = DE.order_id AND O.org_id = DE.org_id WHERE  1 = 1 AND DE.created_timestamp &gt;= Now() - interval 15 minute AND Upper(PLA.planning_strategy_id) LIKE ''STANDARD%'' AND DE.deselected_order_lines &gt; '0' AND DE.org_id = $orgId;"}'</t>
+  </si>
+  <si>
+    <t>{"alertName":"STANDARD ORDERS DESELECTED DURING WAVING","dataSource":"MAWM","database":{"connection":"MAPRD_NEW","type":"MySQL","uri":"jdbc:{host}:{port}/information_schema"},"email":{"subject":"Splunk Alert: $alertName$","body":"&lt;pre&gt;The alert condition for ''$name$'' was triggered.&lt;br /&gt;&lt;br /&gt;***MSP TO CLEAN UP***&lt;br /&gt;Description: &lt;br /&gt;This alert displays routed orders that were deselected from the WMS wave.  Please call the IT Service Desk immediately to correct this condition.  &lt;br /&gt;&lt;br /&gt;Phone: 866-RNDC-HLP (866-763-2457)&lt;/pre&gt;","fromEmail":"wms-tools-noreply@rndc-usa.com","toEmail":"Frank.Ryan@RNDC-USA.COM, David.Gould2@rndc-usa.com, Don.Hamlin@RNDC-USA.COM","ccEmail":"wmsinternal@rndc-usa.com,wmsconsultant@rndc-usa.com   , WMSMSPSupport@RNDC-USA.COM","footer":"","attachment":["link-to-alert","link-to-results","inline-table","attach-csv"]},"sql":"SELECT DE.org_id, DE.order_id, O.ext_route_id, DE.order_planning_run_id, DE.deselected_orders, DE.deselected_order_lines, DE.updated_by, DE.created_timestamp FROM   default_dcorder.DCO_PLAN_RUN_DESELECT_COUNT DE join default_dcorder.DCO_ORDER_PLAN_RUN_STRATEGY PLA ON DE.order_planning_run_id = PLA.order_planning_run_id AND PLA.org_id = DE.org_id left join default_dcorder.DCO_ORDER O ON O.order_id = DE.order_id AND O.org_id = DE.org_id WHERE  1 = 1 AND DE.created_timestamp &gt;= Now() - interval 15 minute AND Upper(PLA.planning_strategy_id) LIKE ''STANDARD%%'' AND DE.deselected_order_lines &gt; ''0'' AND DE.org_id = $orgId;"}'</t>
+  </si>
+  <si>
+    <t>{"alertName":"STANDARD ORDERS DESELECTED DURING WAVING","dataSource":"MAWM","database":{"connection":"MAPRD_NEW","type":"MySQL","uri":"jdbc:{host}:{port}/information_schema"},"email":{"subject":"Splunk Alert: $alertName$","body":"&lt;pre&gt;&lt;br /&gt;The alert condition for ''$name$'' was triggered.&lt;br /&gt;***MSP TO CLEAN UP*** Description: This alert displays routed orders that were deselected from the WMS wave.  Please call the IT Service Desk immediately to correct this condition.  Phone: 866-RNDC-HLP (866-763-2457)&lt;br /&gt;&lt;/pre&gt;","fromEmail":"wms-tools-noreply@rndc-usa.com","toEmail":"bryce.meyer@rndc-usa.com, Michael.Ferdinand@Penske.com, abel.paucardelacruz@rndc-usa.com, Sara.Farrington@Penske.com, Matthew.Chavez@Penske.com,Jesse.Butler@Penske.com, Brian.Bontemps@penske.com","ccEmail":"wmsinternal@RNDC-USA.COM, WMSMSPSupport@RNDC-USA.COM, DL_MANH_RNDC_MAWM_PSO@manh.com, DL_RNDC_MAWM_CSO@manh.com","footer":"","attachment":["link-to-alert","link-to-results","inline-table","attach-csv"]},"sql":"SELECT DE.org_id, DE.order_id, O.ext_route_id, DE.order_planning_run_id, DE.deselected_orders, DE.deselected_order_lines, DE.updated_by, DE.created_timestamp FROM   default_dcorder.DCO_PLAN_RUN_DESELECT_COUNT DE join default_dcorder.DCO_ORDER_PLAN_RUN_STRATEGY PLA ON DE.order_planning_run_id = PLA.order_planning_run_id AND PLA.org_id = DE.org_id left join default_dcorder.DCO_ORDER O ON O.order_id = DE.order_id AND O.org_id = DE.org_id WHERE  1 = 1 AND DE.created_timestamp &gt;= Now() - interval 15 minute AND Upper(PLA.planning_strategy_id) LIKE ''STANDARD%%'' AND DE.deselected_order_lines &gt; ''0'' AND DE.org_id = $orgId;"}'</t>
+  </si>
+  <si>
+    <t>{"alertName":"STANDARD ORDERS DESELECTED DURING WAVING","dataSource":"MAWM","database":{"connection":"MAPRD_NEW","type":"MySQL","uri":"jdbc:{host}:{port}/information_schema"},"email":{"subject":"Splunk Alert: $alertName$","body":"&lt;pre&gt;The alert condition for ''$name$'' was triggered.&lt;/pre&gt;","fromEmail":"wms-tools-noreply@rndc-usa.com","toEmail":"Teppi.Waxman@RNDC-USA.COM, Jesse.Kahalioumi@RNDC-USA.COM, Mark.Carriaga@rndc-usa.com","ccEmail":"wmsinternal@rndc-usa.com, wmsconsultant@rndc-usa.com, WMSMSPSupport@RNDC-USA.COM","footer":"","attachment":["link-to-alert","link-to-results","inline-table"]},"sql":"SELECT DE.org_id, DE.order_id, O.ext_route_id, DE.order_planning_run_id, DE.deselected_orders, DE.deselected_order_lines, DE.updated_by, DE.created_timestamp FROM   default_dcorder.DCO_PLAN_RUN_DESELECT_COUNT DE join default_dcorder.DCO_ORDER_PLAN_RUN_STRATEGY PLA ON DE.order_planning_run_id = PLA.order_planning_run_id AND PLA.org_id = DE.org_id left join default_dcorder.DCO_ORDER O ON O.order_id = DE.order_id AND O.org_id = DE.org_id WHERE  1 = 1 AND DE.created_timestamp &gt;= Now() - interval 15 minute AND Upper(PLA.planning_strategy_id) LIKE ''STANDARD%%'' AND DE.deselected_order_lines &gt; ''0'' AND DE.org_id = $orgId;"}'</t>
+  </si>
+  <si>
+    <t>{"alertName":"STANDARD ORDERS DESELECTED DURING WAVING","dataSource":"MAWM","database":{"connection":"MAPRD_NEW","type":"MySQL","uri":"jdbc:{host}:{port}/information_schema"},"email":{"subject":"Splunk Alert: $alertName$","body":"&lt;pre&gt;The alert condition for ''$name$'' was triggered.&lt;/pre&gt;","fromEmail":"wms-tools-noreply@rndc-usa.com","toEmail":"wmsinternal@RNDC-USA.COM, WMSadmin@RNDC-USA.COM, WMSMSPSupport@RNDC-USA.COM","ccEmail":"","footer":"","attachment":["link-to-alert","link-to-results","inline-table"]},"sql":"SELECT DE.org_id, DE.order_id, O.ext_route_id, DE.order_planning_run_id, DE.deselected_orders, DE.deselected_order_lines, DE.updated_by, DE.created_timestamp FROM   default_dcorder.DCO_PLAN_RUN_DESELECT_COUNT DE join default_dcorder.DCO_ORDER_PLAN_RUN_STRATEGY PLA ON DE.order_planning_run_id = PLA.order_planning_run_id AND PLA.org_id = DE.org_id left join default_dcorder.DCO_ORDER O ON O.order_id = DE.order_id AND O.org_id = DE.org_id WHERE  1 = 1 AND DE.created_timestamp &gt;= Now() - interval 15 minute AND Upper(PLA.planning_strategy_id) LIKE ''STANDARD%%'' AND DE.deselected_order_lines &gt; ''0'' AND DE.org_id = $orgId;"}'</t>
+  </si>
+  <si>
+    <t>{"alertName":"STANDARD ORDERS DESELECTED DURING WAVING","dataSource":"MAWM","database":{"connection":"MAPRD_NEW","type":"MySQL","uri":"jdbc:{host}:{port}/information_schema"},"email":{"subject":"Splunk Alert: $alertName$","body":"&lt;pre&gt;The alert condition for ''$name$'' was triggered.&lt;br /&gt;&lt;br /&gt;***MSP TO CLEAN UP***&lt;br /&gt;Description: &lt;br /&gt;This alert displays routed orders that were deselected from the WMS wave.  Please call the IT Service Desk immediately to correct this condition.  &lt;br /&gt;&lt;br /&gt;Phone: 866-RNDC-HLP (866-763-2457)&lt;/pre&gt;","fromEmail":"wms-tools-noreply@rndc-usa.com","toEmail":"ryan.mchenry@rndc-usa.com,franco.flores@rndc-usa.com,McHenry@rndc-usa.com,BENJAMIN.SUTTON@RNDC-USA.COM,Antonio.Larez@RNDC-USA.COM,wmsinternal@RNDC-USA.COM, DL_MANH_RNDC_MAWM_PSO@manh.com, DL_RNDC_MAWM_CSO@manh.com","ccEmail":"wmsinternal@rndc-usa.com, wmsconsultant@rndc-usa.com, WMSMSPSupport@RNDC-USA.COM","footer":"","attachment":["link-to-alert","link-to-results","inline-table","attach-csv"]},"sql":"SELECT DE.org_id, DE.order_id, O.ext_route_id, DE.order_planning_run_id, DE.deselected_orders, DE.deselected_order_lines, DE.updated_by, DE.created_timestamp FROM   default_dcorder.DCO_PLAN_RUN_DESELECT_COUNT DE join default_dcorder.DCO_ORDER_PLAN_RUN_STRATEGY PLA ON DE.order_planning_run_id = PLA.order_planning_run_id AND PLA.org_id = DE.org_id left join default_dcorder.DCO_ORDER O ON O.order_id = DE.order_id AND O.org_id = DE.org_id WHERE  1 = 1 AND DE.created_timestamp &gt;= Now() - interval 15 minute AND Upper(PLA.planning_strategy_id) LIKE ''STANDARD%%'' AND DE.deselected_order_lines &gt; ''0'' AND DE.org_id = $orgId;"}'</t>
   </si>
 </sst>
 </file>
@@ -1971,10 +1983,10 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A63BE434-9ED0-E94E-BE21-7A21279D6729}">
-  <dimension ref="A1:L47"/>
+  <dimension ref="A1:L53"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="7" max="7" width="195.33203125" customWidth="1"/>
+    <col min="7" max="7" width="80.83203125" customWidth="1"/>
     <col min="8" max="8" width="17.5" customWidth="1"/>
   </cols>
   <sheetData>
@@ -2013,259 +2025,259 @@
         <v>171</v>
       </c>
     </row>
-    <row r="2" spans="1:12" ht="17" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:12" ht="372" x14ac:dyDescent="0.2">
       <c r="A2" t="b">
         <v>0</v>
       </c>
       <c r="B2" s="3" t="s">
+        <v>176</v>
+      </c>
+      <c r="C2" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="D2" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="E2">
+        <v>2</v>
+      </c>
+      <c r="F2" s="3" t="s">
         <v>177</v>
       </c>
-      <c r="C2" s="3" t="s">
+      <c r="G2" s="13" t="s">
+        <v>184</v>
+      </c>
+      <c r="H2" s="3" t="s">
+        <v>172</v>
+      </c>
+      <c r="I2" s="3" t="s">
+        <v>173</v>
+      </c>
+      <c r="J2" s="3" t="s">
+        <v>172</v>
+      </c>
+      <c r="K2" s="3" t="s">
+        <v>173</v>
+      </c>
+      <c r="L2" s="12"/>
+    </row>
+    <row r="3" spans="1:12" ht="255" x14ac:dyDescent="0.2">
+      <c r="A3" t="b">
+        <v>0</v>
+      </c>
+      <c r="B3" s="3" t="s">
+        <v>176</v>
+      </c>
+      <c r="C3" s="3" t="s">
+        <v>35</v>
+      </c>
+      <c r="D3" s="3" t="s">
+        <v>35</v>
+      </c>
+      <c r="E3">
+        <v>27</v>
+      </c>
+      <c r="F3" s="3" t="s">
+        <v>177</v>
+      </c>
+      <c r="G3" s="13" t="s">
+        <v>183</v>
+      </c>
+      <c r="H3" s="3" t="s">
+        <v>172</v>
+      </c>
+      <c r="I3" s="3" t="s">
+        <v>173</v>
+      </c>
+      <c r="J3" s="3" t="s">
+        <v>172</v>
+      </c>
+      <c r="K3" s="3" t="s">
+        <v>173</v>
+      </c>
+    </row>
+    <row r="4" spans="1:12" ht="372" x14ac:dyDescent="0.2">
+      <c r="A4" t="b">
+        <v>0</v>
+      </c>
+      <c r="B4" s="3" t="s">
+        <v>176</v>
+      </c>
+      <c r="C4" s="3" t="s">
         <v>13</v>
       </c>
-      <c r="D2" s="3" t="s">
+      <c r="D4" s="3" t="s">
         <v>13</v>
       </c>
-      <c r="E2">
+      <c r="E4">
         <v>3</v>
       </c>
-      <c r="F2" s="3" t="s">
-        <v>178</v>
-      </c>
-      <c r="G2" s="13" t="s">
+      <c r="F4" s="3" t="s">
+        <v>177</v>
+      </c>
+      <c r="G4" s="13" t="s">
+        <v>184</v>
+      </c>
+      <c r="H4" s="3" t="s">
+        <v>172</v>
+      </c>
+      <c r="I4" s="3" t="s">
+        <v>173</v>
+      </c>
+      <c r="J4" s="3" t="s">
+        <v>172</v>
+      </c>
+      <c r="K4" s="3" t="s">
+        <v>173</v>
+      </c>
+      <c r="L4" s="3"/>
+    </row>
+    <row r="5" spans="1:12" ht="255" x14ac:dyDescent="0.2">
+      <c r="A5" t="b">
+        <v>0</v>
+      </c>
+      <c r="B5" s="3" t="s">
         <v>176</v>
       </c>
-      <c r="H2" s="3" t="s">
-        <v>172</v>
-      </c>
-      <c r="I2" s="3" t="s">
-        <v>173</v>
-      </c>
-      <c r="J2" s="3" t="s">
-        <v>172</v>
-      </c>
-      <c r="K2" s="3" t="s">
-        <v>173</v>
-      </c>
-      <c r="L2" s="12"/>
-    </row>
-    <row r="3" spans="1:12" ht="17" x14ac:dyDescent="0.2">
-      <c r="A3" t="b">
-        <v>0</v>
-      </c>
-      <c r="B3" s="3" t="s">
+      <c r="C5" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="D5" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="E5">
+        <v>4</v>
+      </c>
+      <c r="F5" s="3" t="s">
         <v>177</v>
       </c>
-      <c r="C3" s="3" t="s">
-        <v>8</v>
-      </c>
-      <c r="D3" s="3" t="s">
-        <v>8</v>
-      </c>
-      <c r="E3">
-        <v>4</v>
-      </c>
-      <c r="F3" s="3" t="s">
-        <v>178</v>
-      </c>
-      <c r="G3" s="13" t="s">
+      <c r="G5" s="13" t="s">
+        <v>183</v>
+      </c>
+      <c r="H5" s="3" t="s">
+        <v>172</v>
+      </c>
+      <c r="I5" s="3" t="s">
+        <v>173</v>
+      </c>
+      <c r="J5" s="3" t="s">
+        <v>172</v>
+      </c>
+      <c r="K5" s="3" t="s">
+        <v>173</v>
+      </c>
+    </row>
+    <row r="6" spans="1:12" ht="255" x14ac:dyDescent="0.2">
+      <c r="A6" t="b">
+        <v>0</v>
+      </c>
+      <c r="B6" s="3" t="s">
         <v>176</v>
       </c>
-      <c r="H3" s="3" t="s">
-        <v>172</v>
-      </c>
-      <c r="I3" s="3" t="s">
-        <v>173</v>
-      </c>
-      <c r="J3" s="3" t="s">
-        <v>172</v>
-      </c>
-      <c r="K3" s="3" t="s">
-        <v>173</v>
-      </c>
-    </row>
-    <row r="4" spans="1:12" ht="17" x14ac:dyDescent="0.2">
-      <c r="A4" t="b">
-        <v>0</v>
-      </c>
-      <c r="B4" s="3" t="s">
+      <c r="C6" t="s">
+        <v>36</v>
+      </c>
+      <c r="D6" t="s">
+        <v>36</v>
+      </c>
+      <c r="E6">
+        <v>28</v>
+      </c>
+      <c r="F6" s="3" t="s">
         <v>177</v>
       </c>
-      <c r="C4" s="3" t="s">
-        <v>9</v>
-      </c>
-      <c r="D4" s="3" t="s">
-        <v>9</v>
-      </c>
-      <c r="E4">
-        <v>21</v>
-      </c>
-      <c r="F4" s="3" t="s">
-        <v>178</v>
-      </c>
-      <c r="G4" s="13" t="s">
+      <c r="G6" s="13" t="s">
+        <v>183</v>
+      </c>
+      <c r="H6" s="3" t="s">
+        <v>172</v>
+      </c>
+      <c r="I6" s="3" t="s">
+        <v>173</v>
+      </c>
+      <c r="J6" s="3" t="s">
+        <v>172</v>
+      </c>
+      <c r="K6" s="3" t="s">
+        <v>173</v>
+      </c>
+    </row>
+    <row r="7" spans="1:12" ht="255" x14ac:dyDescent="0.2">
+      <c r="A7" t="b">
+        <v>0</v>
+      </c>
+      <c r="B7" s="3" t="s">
         <v>176</v>
       </c>
-      <c r="H4" s="3" t="s">
-        <v>172</v>
-      </c>
-      <c r="I4" s="3" t="s">
-        <v>173</v>
-      </c>
-      <c r="J4" s="3" t="s">
-        <v>172</v>
-      </c>
-      <c r="K4" s="3" t="s">
-        <v>173</v>
-      </c>
-      <c r="L4" s="3"/>
-    </row>
-    <row r="5" spans="1:12" ht="17" x14ac:dyDescent="0.2">
-      <c r="A5" t="b">
-        <v>0</v>
-      </c>
-      <c r="B5" s="3" t="s">
+      <c r="C7" t="s">
+        <v>47</v>
+      </c>
+      <c r="D7" t="s">
+        <v>47</v>
+      </c>
+      <c r="E7">
+        <v>39</v>
+      </c>
+      <c r="F7" s="3" t="s">
         <v>177</v>
       </c>
-      <c r="C5" s="3" t="s">
-        <v>30</v>
-      </c>
-      <c r="D5" s="3" t="s">
-        <v>30</v>
-      </c>
-      <c r="E5">
-        <v>22</v>
-      </c>
-      <c r="F5" s="3" t="s">
-        <v>178</v>
-      </c>
-      <c r="G5" s="13" t="s">
+      <c r="G7" s="13" t="s">
+        <v>183</v>
+      </c>
+      <c r="H7" s="3" t="s">
+        <v>172</v>
+      </c>
+      <c r="I7" s="3" t="s">
+        <v>173</v>
+      </c>
+      <c r="J7" s="3" t="s">
+        <v>172</v>
+      </c>
+      <c r="K7" s="3" t="s">
+        <v>173</v>
+      </c>
+    </row>
+    <row r="8" spans="1:12" ht="255" x14ac:dyDescent="0.2">
+      <c r="A8" t="b">
+        <v>0</v>
+      </c>
+      <c r="B8" s="3" t="s">
         <v>176</v>
       </c>
-      <c r="H5" s="3" t="s">
-        <v>172</v>
-      </c>
-      <c r="I5" s="3" t="s">
-        <v>173</v>
-      </c>
-      <c r="J5" s="3" t="s">
-        <v>172</v>
-      </c>
-      <c r="K5" s="3" t="s">
-        <v>173</v>
-      </c>
-    </row>
-    <row r="6" spans="1:12" ht="17" x14ac:dyDescent="0.2">
-      <c r="A6" t="b">
-        <v>0</v>
-      </c>
-      <c r="B6" s="3" t="s">
+      <c r="C8" t="s">
+        <v>49</v>
+      </c>
+      <c r="D8" t="s">
+        <v>49</v>
+      </c>
+      <c r="E8">
+        <v>41</v>
+      </c>
+      <c r="F8" s="3" t="s">
         <v>177</v>
       </c>
-      <c r="C6" s="3" t="s">
-        <v>35</v>
-      </c>
-      <c r="D6" s="3" t="s">
-        <v>35</v>
-      </c>
-      <c r="E6">
-        <v>27</v>
-      </c>
-      <c r="F6" s="3" t="s">
-        <v>178</v>
-      </c>
-      <c r="G6" s="13" t="s">
+      <c r="G8" s="13" t="s">
+        <v>183</v>
+      </c>
+      <c r="H8" s="3" t="s">
+        <v>172</v>
+      </c>
+      <c r="I8" s="3" t="s">
+        <v>173</v>
+      </c>
+      <c r="J8" s="3" t="s">
+        <v>172</v>
+      </c>
+      <c r="K8" s="3" t="s">
+        <v>173</v>
+      </c>
+    </row>
+    <row r="9" spans="1:12" ht="255" x14ac:dyDescent="0.2">
+      <c r="A9" t="b">
+        <v>0</v>
+      </c>
+      <c r="B9" s="3" t="s">
         <v>176</v>
-      </c>
-      <c r="H6" s="3" t="s">
-        <v>172</v>
-      </c>
-      <c r="I6" s="3" t="s">
-        <v>173</v>
-      </c>
-      <c r="J6" s="3" t="s">
-        <v>172</v>
-      </c>
-      <c r="K6" s="3" t="s">
-        <v>173</v>
-      </c>
-    </row>
-    <row r="7" spans="1:12" ht="17" x14ac:dyDescent="0.2">
-      <c r="A7" t="b">
-        <v>0</v>
-      </c>
-      <c r="B7" s="3" t="s">
-        <v>177</v>
-      </c>
-      <c r="C7" s="3" t="s">
-        <v>37</v>
-      </c>
-      <c r="D7" s="3" t="s">
-        <v>37</v>
-      </c>
-      <c r="E7">
-        <v>29</v>
-      </c>
-      <c r="F7" s="3" t="s">
-        <v>178</v>
-      </c>
-      <c r="G7" s="13" t="s">
-        <v>176</v>
-      </c>
-      <c r="H7" s="3" t="s">
-        <v>172</v>
-      </c>
-      <c r="I7" s="3" t="s">
-        <v>173</v>
-      </c>
-      <c r="J7" s="3" t="s">
-        <v>172</v>
-      </c>
-      <c r="K7" s="3" t="s">
-        <v>173</v>
-      </c>
-    </row>
-    <row r="8" spans="1:12" ht="17" x14ac:dyDescent="0.2">
-      <c r="A8" t="b">
-        <v>0</v>
-      </c>
-      <c r="B8" s="3" t="s">
-        <v>177</v>
-      </c>
-      <c r="C8" s="3" t="s">
-        <v>39</v>
-      </c>
-      <c r="D8" s="3" t="s">
-        <v>39</v>
-      </c>
-      <c r="E8">
-        <v>31</v>
-      </c>
-      <c r="F8" s="3" t="s">
-        <v>178</v>
-      </c>
-      <c r="G8" s="13" t="s">
-        <v>176</v>
-      </c>
-      <c r="H8" s="3" t="s">
-        <v>172</v>
-      </c>
-      <c r="I8" s="3" t="s">
-        <v>173</v>
-      </c>
-      <c r="J8" s="3" t="s">
-        <v>172</v>
-      </c>
-      <c r="K8" s="3" t="s">
-        <v>173</v>
-      </c>
-    </row>
-    <row r="9" spans="1:12" ht="17" x14ac:dyDescent="0.2">
-      <c r="A9" t="b">
-        <v>0</v>
-      </c>
-      <c r="B9" s="3" t="s">
-        <v>177</v>
       </c>
       <c r="C9" s="3" t="s">
         <v>50</v>
@@ -2277,275 +2289,275 @@
         <v>42</v>
       </c>
       <c r="F9" s="3" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
       <c r="G9" s="13" t="s">
+        <v>183</v>
+      </c>
+      <c r="H9" s="3" t="s">
+        <v>172</v>
+      </c>
+      <c r="I9" s="3" t="s">
+        <v>173</v>
+      </c>
+      <c r="J9" s="3" t="s">
+        <v>172</v>
+      </c>
+      <c r="K9" s="3" t="s">
+        <v>173</v>
+      </c>
+    </row>
+    <row r="10" spans="1:12" ht="255" x14ac:dyDescent="0.2">
+      <c r="A10" t="b">
+        <v>0</v>
+      </c>
+      <c r="B10" s="3" t="s">
         <v>176</v>
       </c>
-      <c r="H9" s="3" t="s">
-        <v>172</v>
-      </c>
-      <c r="I9" s="3" t="s">
-        <v>173</v>
-      </c>
-      <c r="J9" s="3" t="s">
-        <v>172</v>
-      </c>
-      <c r="K9" s="3" t="s">
-        <v>173</v>
-      </c>
-    </row>
-    <row r="10" spans="1:12" ht="17" x14ac:dyDescent="0.2">
-      <c r="A10" t="b">
-        <v>0</v>
-      </c>
-      <c r="B10" s="3" t="s">
+      <c r="C10" t="s">
+        <v>14</v>
+      </c>
+      <c r="D10" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="E10">
+        <v>5</v>
+      </c>
+      <c r="F10" s="3" t="s">
         <v>177</v>
       </c>
-      <c r="C10" s="3" t="s">
-        <v>12</v>
-      </c>
-      <c r="D10" s="3" t="s">
-        <v>12</v>
-      </c>
-      <c r="E10">
-        <v>2</v>
-      </c>
-      <c r="F10" s="3" t="s">
-        <v>178</v>
-      </c>
       <c r="G10" s="13" t="s">
+        <v>183</v>
+      </c>
+      <c r="H10" s="3" t="s">
+        <v>172</v>
+      </c>
+      <c r="I10" s="3" t="s">
+        <v>173</v>
+      </c>
+      <c r="J10" s="3" t="s">
+        <v>172</v>
+      </c>
+      <c r="K10" s="3" t="s">
+        <v>173</v>
+      </c>
+    </row>
+    <row r="11" spans="1:12" ht="372" x14ac:dyDescent="0.2">
+      <c r="A11" t="b">
+        <v>0</v>
+      </c>
+      <c r="B11" s="3" t="s">
         <v>176</v>
       </c>
-      <c r="H10" s="3" t="s">
-        <v>172</v>
-      </c>
-      <c r="I10" s="3" t="s">
-        <v>173</v>
-      </c>
-      <c r="J10" s="3" t="s">
-        <v>172</v>
-      </c>
-      <c r="K10" s="3" t="s">
-        <v>173</v>
-      </c>
-    </row>
-    <row r="11" spans="1:12" ht="17" x14ac:dyDescent="0.2">
-      <c r="A11" t="b">
-        <v>0</v>
-      </c>
-      <c r="B11" s="3" t="s">
+      <c r="C11" t="s">
+        <v>15</v>
+      </c>
+      <c r="D11" t="s">
+        <v>15</v>
+      </c>
+      <c r="E11">
+        <v>6</v>
+      </c>
+      <c r="F11" s="3" t="s">
         <v>177</v>
       </c>
-      <c r="C11" t="s">
-        <v>14</v>
-      </c>
-      <c r="D11" s="3" t="s">
-        <v>14</v>
-      </c>
-      <c r="E11">
-        <v>5</v>
-      </c>
-      <c r="F11" s="3" t="s">
-        <v>178</v>
-      </c>
       <c r="G11" s="13" t="s">
+        <v>184</v>
+      </c>
+      <c r="H11" s="3" t="s">
+        <v>172</v>
+      </c>
+      <c r="I11" s="3" t="s">
+        <v>173</v>
+      </c>
+      <c r="J11" s="3" t="s">
+        <v>172</v>
+      </c>
+      <c r="K11" s="3" t="s">
+        <v>173</v>
+      </c>
+    </row>
+    <row r="12" spans="1:12" ht="136" x14ac:dyDescent="0.2">
+      <c r="A12" t="b">
+        <v>0</v>
+      </c>
+      <c r="B12" s="3" t="s">
         <v>176</v>
       </c>
-      <c r="H11" s="3" t="s">
-        <v>172</v>
-      </c>
-      <c r="I11" s="3" t="s">
-        <v>173</v>
-      </c>
-      <c r="J11" s="3" t="s">
-        <v>172</v>
-      </c>
-      <c r="K11" s="3" t="s">
-        <v>173</v>
-      </c>
-    </row>
-    <row r="12" spans="1:12" ht="17" x14ac:dyDescent="0.2">
-      <c r="A12" t="b">
-        <v>0</v>
-      </c>
-      <c r="B12" s="3" t="s">
+      <c r="C12" t="s">
+        <v>16</v>
+      </c>
+      <c r="D12" t="s">
+        <v>16</v>
+      </c>
+      <c r="E12">
+        <v>7</v>
+      </c>
+      <c r="F12" s="3" t="s">
         <v>177</v>
       </c>
-      <c r="C12" t="s">
-        <v>15</v>
-      </c>
-      <c r="D12" t="s">
-        <v>15</v>
-      </c>
-      <c r="E12">
-        <v>6</v>
-      </c>
-      <c r="F12" s="3" t="s">
-        <v>178</v>
-      </c>
       <c r="G12" s="13" t="s">
+        <v>180</v>
+      </c>
+      <c r="H12" s="3" t="s">
+        <v>172</v>
+      </c>
+      <c r="I12" s="3" t="s">
+        <v>173</v>
+      </c>
+      <c r="J12" s="3" t="s">
+        <v>172</v>
+      </c>
+      <c r="K12" s="3" t="s">
+        <v>173</v>
+      </c>
+    </row>
+    <row r="13" spans="1:12" ht="255" x14ac:dyDescent="0.2">
+      <c r="A13" t="b">
+        <v>0</v>
+      </c>
+      <c r="B13" s="3" t="s">
         <v>176</v>
       </c>
-      <c r="H12" s="3" t="s">
-        <v>172</v>
-      </c>
-      <c r="I12" s="3" t="s">
-        <v>173</v>
-      </c>
-      <c r="J12" s="3" t="s">
-        <v>172</v>
-      </c>
-      <c r="K12" s="3" t="s">
-        <v>173</v>
-      </c>
-    </row>
-    <row r="13" spans="1:12" ht="17" x14ac:dyDescent="0.2">
-      <c r="A13" t="b">
-        <v>0</v>
-      </c>
-      <c r="B13" s="3" t="s">
+      <c r="C13" t="s">
+        <v>17</v>
+      </c>
+      <c r="D13" t="s">
+        <v>17</v>
+      </c>
+      <c r="E13">
+        <v>8</v>
+      </c>
+      <c r="F13" s="3" t="s">
         <v>177</v>
       </c>
-      <c r="C13" t="s">
-        <v>16</v>
-      </c>
-      <c r="D13" t="s">
-        <v>16</v>
-      </c>
-      <c r="E13">
-        <v>7</v>
-      </c>
-      <c r="F13" s="3" t="s">
-        <v>178</v>
-      </c>
       <c r="G13" s="13" t="s">
+        <v>183</v>
+      </c>
+      <c r="H13" s="3" t="s">
+        <v>172</v>
+      </c>
+      <c r="I13" s="3" t="s">
+        <v>173</v>
+      </c>
+      <c r="J13" s="3" t="s">
+        <v>172</v>
+      </c>
+      <c r="K13" s="3" t="s">
+        <v>173</v>
+      </c>
+    </row>
+    <row r="14" spans="1:12" ht="255" x14ac:dyDescent="0.2">
+      <c r="A14" t="b">
+        <v>0</v>
+      </c>
+      <c r="B14" s="3" t="s">
         <v>176</v>
       </c>
-      <c r="H13" s="3" t="s">
-        <v>172</v>
-      </c>
-      <c r="I13" s="3" t="s">
-        <v>173</v>
-      </c>
-      <c r="J13" s="3" t="s">
-        <v>172</v>
-      </c>
-      <c r="K13" s="3" t="s">
-        <v>173</v>
-      </c>
-    </row>
-    <row r="14" spans="1:12" ht="17" x14ac:dyDescent="0.2">
-      <c r="A14" t="b">
-        <v>0</v>
-      </c>
-      <c r="B14" s="3" t="s">
+      <c r="C14" t="s">
+        <v>18</v>
+      </c>
+      <c r="D14" t="s">
+        <v>18</v>
+      </c>
+      <c r="E14">
+        <v>9</v>
+      </c>
+      <c r="F14" s="3" t="s">
         <v>177</v>
       </c>
-      <c r="C14" t="s">
-        <v>17</v>
-      </c>
-      <c r="D14" t="s">
-        <v>17</v>
-      </c>
-      <c r="E14">
-        <v>8</v>
-      </c>
-      <c r="F14" s="3" t="s">
-        <v>178</v>
-      </c>
       <c r="G14" s="13" t="s">
+        <v>183</v>
+      </c>
+      <c r="H14" s="3" t="s">
+        <v>172</v>
+      </c>
+      <c r="I14" s="3" t="s">
+        <v>173</v>
+      </c>
+      <c r="J14" s="3" t="s">
+        <v>172</v>
+      </c>
+      <c r="K14" s="3" t="s">
+        <v>173</v>
+      </c>
+    </row>
+    <row r="15" spans="1:12" ht="255" x14ac:dyDescent="0.2">
+      <c r="A15" t="b">
+        <v>0</v>
+      </c>
+      <c r="B15" s="3" t="s">
         <v>176</v>
       </c>
-      <c r="H14" s="3" t="s">
-        <v>172</v>
-      </c>
-      <c r="I14" s="3" t="s">
-        <v>173</v>
-      </c>
-      <c r="J14" s="3" t="s">
-        <v>172</v>
-      </c>
-      <c r="K14" s="3" t="s">
-        <v>173</v>
-      </c>
-    </row>
-    <row r="15" spans="1:12" ht="17" x14ac:dyDescent="0.2">
-      <c r="A15" t="b">
-        <v>0</v>
-      </c>
-      <c r="B15" s="3" t="s">
+      <c r="C15" t="s">
+        <v>19</v>
+      </c>
+      <c r="D15" t="s">
+        <v>19</v>
+      </c>
+      <c r="E15">
+        <v>10</v>
+      </c>
+      <c r="F15" s="3" t="s">
         <v>177</v>
       </c>
-      <c r="C15" t="s">
-        <v>18</v>
-      </c>
-      <c r="D15" t="s">
-        <v>18</v>
-      </c>
-      <c r="E15">
-        <v>9</v>
-      </c>
-      <c r="F15" s="3" t="s">
-        <v>178</v>
-      </c>
       <c r="G15" s="13" t="s">
+        <v>183</v>
+      </c>
+      <c r="H15" s="3" t="s">
+        <v>172</v>
+      </c>
+      <c r="I15" s="3" t="s">
+        <v>173</v>
+      </c>
+      <c r="J15" s="3" t="s">
+        <v>172</v>
+      </c>
+      <c r="K15" s="3" t="s">
+        <v>173</v>
+      </c>
+    </row>
+    <row r="16" spans="1:12" ht="102" x14ac:dyDescent="0.2">
+      <c r="A16" t="b">
+        <v>0</v>
+      </c>
+      <c r="B16" s="3" t="s">
         <v>176</v>
       </c>
-      <c r="H15" s="3" t="s">
-        <v>172</v>
-      </c>
-      <c r="I15" s="3" t="s">
-        <v>173</v>
-      </c>
-      <c r="J15" s="3" t="s">
-        <v>172</v>
-      </c>
-      <c r="K15" s="3" t="s">
-        <v>173</v>
-      </c>
-    </row>
-    <row r="16" spans="1:12" ht="17" x14ac:dyDescent="0.2">
-      <c r="A16" t="b">
-        <v>0</v>
-      </c>
-      <c r="B16" s="3" t="s">
+      <c r="C16" t="s">
+        <v>44</v>
+      </c>
+      <c r="D16" t="s">
+        <v>44</v>
+      </c>
+      <c r="E16">
+        <v>36</v>
+      </c>
+      <c r="F16" s="3" t="s">
         <v>177</v>
       </c>
-      <c r="C16" t="s">
-        <v>19</v>
-      </c>
-      <c r="D16" t="s">
-        <v>19</v>
-      </c>
-      <c r="E16">
-        <v>10</v>
-      </c>
-      <c r="F16" s="3" t="s">
-        <v>178</v>
-      </c>
       <c r="G16" s="13" t="s">
+        <v>182</v>
+      </c>
+      <c r="H16" s="3" t="s">
+        <v>172</v>
+      </c>
+      <c r="I16" s="3" t="s">
+        <v>173</v>
+      </c>
+      <c r="J16" s="3" t="s">
+        <v>172</v>
+      </c>
+      <c r="K16" s="3" t="s">
+        <v>173</v>
+      </c>
+    </row>
+    <row r="17" spans="1:11" ht="255" x14ac:dyDescent="0.2">
+      <c r="A17" t="b">
+        <v>0</v>
+      </c>
+      <c r="B17" s="3" t="s">
         <v>176</v>
-      </c>
-      <c r="H16" s="3" t="s">
-        <v>172</v>
-      </c>
-      <c r="I16" s="3" t="s">
-        <v>173</v>
-      </c>
-      <c r="J16" s="3" t="s">
-        <v>172</v>
-      </c>
-      <c r="K16" s="3" t="s">
-        <v>173</v>
-      </c>
-    </row>
-    <row r="17" spans="1:11" ht="17" x14ac:dyDescent="0.2">
-      <c r="A17" t="b">
-        <v>0</v>
-      </c>
-      <c r="B17" s="3" t="s">
-        <v>177</v>
       </c>
       <c r="C17" t="s">
         <v>20</v>
@@ -2557,30 +2569,30 @@
         <v>11</v>
       </c>
       <c r="F17" s="3" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
       <c r="G17" s="13" t="s">
+        <v>183</v>
+      </c>
+      <c r="H17" s="3" t="s">
+        <v>172</v>
+      </c>
+      <c r="I17" s="3" t="s">
+        <v>173</v>
+      </c>
+      <c r="J17" s="3" t="s">
+        <v>172</v>
+      </c>
+      <c r="K17" s="3" t="s">
+        <v>173</v>
+      </c>
+    </row>
+    <row r="18" spans="1:11" ht="306" x14ac:dyDescent="0.2">
+      <c r="A18" t="b">
+        <v>0</v>
+      </c>
+      <c r="B18" s="3" t="s">
         <v>176</v>
-      </c>
-      <c r="H17" s="3" t="s">
-        <v>172</v>
-      </c>
-      <c r="I17" s="3" t="s">
-        <v>173</v>
-      </c>
-      <c r="J17" s="3" t="s">
-        <v>172</v>
-      </c>
-      <c r="K17" s="3" t="s">
-        <v>173</v>
-      </c>
-    </row>
-    <row r="18" spans="1:11" ht="17" x14ac:dyDescent="0.2">
-      <c r="A18" t="b">
-        <v>0</v>
-      </c>
-      <c r="B18" s="3" t="s">
-        <v>177</v>
       </c>
       <c r="C18" t="s">
         <v>21</v>
@@ -2592,30 +2604,30 @@
         <v>12</v>
       </c>
       <c r="F18" s="3" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
       <c r="G18" s="13" t="s">
+        <v>180</v>
+      </c>
+      <c r="H18" s="3" t="s">
+        <v>172</v>
+      </c>
+      <c r="I18" s="3" t="s">
+        <v>173</v>
+      </c>
+      <c r="J18" s="3" t="s">
+        <v>172</v>
+      </c>
+      <c r="K18" s="3" t="s">
+        <v>173</v>
+      </c>
+    </row>
+    <row r="19" spans="1:11" ht="255" x14ac:dyDescent="0.2">
+      <c r="A19" t="b">
+        <v>0</v>
+      </c>
+      <c r="B19" s="3" t="s">
         <v>176</v>
-      </c>
-      <c r="H18" s="3" t="s">
-        <v>172</v>
-      </c>
-      <c r="I18" s="3" t="s">
-        <v>173</v>
-      </c>
-      <c r="J18" s="3" t="s">
-        <v>172</v>
-      </c>
-      <c r="K18" s="3" t="s">
-        <v>173</v>
-      </c>
-    </row>
-    <row r="19" spans="1:11" ht="17" x14ac:dyDescent="0.2">
-      <c r="A19" t="b">
-        <v>0</v>
-      </c>
-      <c r="B19" s="3" t="s">
-        <v>177</v>
       </c>
       <c r="C19" t="s">
         <v>22</v>
@@ -2627,30 +2639,30 @@
         <v>13</v>
       </c>
       <c r="F19" s="3" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
       <c r="G19" s="13" t="s">
+        <v>183</v>
+      </c>
+      <c r="H19" s="3" t="s">
+        <v>172</v>
+      </c>
+      <c r="I19" s="3" t="s">
+        <v>173</v>
+      </c>
+      <c r="J19" s="3" t="s">
+        <v>172</v>
+      </c>
+      <c r="K19" s="3" t="s">
+        <v>173</v>
+      </c>
+    </row>
+    <row r="20" spans="1:11" ht="255" x14ac:dyDescent="0.2">
+      <c r="A20" t="b">
+        <v>0</v>
+      </c>
+      <c r="B20" s="3" t="s">
         <v>176</v>
-      </c>
-      <c r="H19" s="3" t="s">
-        <v>172</v>
-      </c>
-      <c r="I19" s="3" t="s">
-        <v>173</v>
-      </c>
-      <c r="J19" s="3" t="s">
-        <v>172</v>
-      </c>
-      <c r="K19" s="3" t="s">
-        <v>173</v>
-      </c>
-    </row>
-    <row r="20" spans="1:11" ht="17" x14ac:dyDescent="0.2">
-      <c r="A20" t="b">
-        <v>0</v>
-      </c>
-      <c r="B20" s="3" t="s">
-        <v>177</v>
       </c>
       <c r="C20" t="s">
         <v>23</v>
@@ -2662,535 +2674,535 @@
         <v>14</v>
       </c>
       <c r="F20" s="3" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
       <c r="G20" s="13" t="s">
+        <v>183</v>
+      </c>
+      <c r="H20" s="3" t="s">
+        <v>172</v>
+      </c>
+      <c r="I20" s="3" t="s">
+        <v>173</v>
+      </c>
+      <c r="J20" s="3" t="s">
+        <v>172</v>
+      </c>
+      <c r="K20" s="3" t="s">
+        <v>173</v>
+      </c>
+    </row>
+    <row r="21" spans="1:11" ht="272" x14ac:dyDescent="0.2">
+      <c r="A21" t="b">
+        <v>0</v>
+      </c>
+      <c r="B21" s="3" t="s">
         <v>176</v>
       </c>
-      <c r="H20" s="3" t="s">
-        <v>172</v>
-      </c>
-      <c r="I20" s="3" t="s">
-        <v>173</v>
-      </c>
-      <c r="J20" s="3" t="s">
-        <v>172</v>
-      </c>
-      <c r="K20" s="3" t="s">
-        <v>173</v>
-      </c>
-    </row>
-    <row r="21" spans="1:11" ht="17" x14ac:dyDescent="0.2">
-      <c r="A21" t="b">
-        <v>0</v>
-      </c>
-      <c r="B21" s="3" t="s">
+      <c r="C21" t="s">
+        <v>41</v>
+      </c>
+      <c r="D21" t="s">
+        <v>41</v>
+      </c>
+      <c r="E21">
+        <v>33</v>
+      </c>
+      <c r="F21" s="3" t="s">
         <v>177</v>
       </c>
-      <c r="C21" t="s">
+      <c r="G21" s="13" t="s">
+        <v>182</v>
+      </c>
+      <c r="H21" s="3" t="s">
+        <v>172</v>
+      </c>
+      <c r="I21" s="3" t="s">
+        <v>173</v>
+      </c>
+      <c r="J21" s="3" t="s">
+        <v>172</v>
+      </c>
+      <c r="K21" s="3" t="s">
+        <v>173</v>
+      </c>
+    </row>
+    <row r="22" spans="1:11" ht="272" x14ac:dyDescent="0.2">
+      <c r="A22" t="b">
+        <v>0</v>
+      </c>
+      <c r="B22" s="3" t="s">
+        <v>176</v>
+      </c>
+      <c r="C22" t="s">
+        <v>43</v>
+      </c>
+      <c r="D22" t="s">
+        <v>43</v>
+      </c>
+      <c r="E22">
+        <v>35</v>
+      </c>
+      <c r="F22" s="3" t="s">
+        <v>177</v>
+      </c>
+      <c r="G22" s="13" t="s">
+        <v>182</v>
+      </c>
+      <c r="H22" s="3" t="s">
+        <v>172</v>
+      </c>
+      <c r="I22" s="3" t="s">
+        <v>173</v>
+      </c>
+      <c r="J22" s="3" t="s">
+        <v>172</v>
+      </c>
+      <c r="K22" s="3" t="s">
+        <v>173</v>
+      </c>
+    </row>
+    <row r="23" spans="1:11" ht="255" x14ac:dyDescent="0.2">
+      <c r="A23" t="b">
+        <v>0</v>
+      </c>
+      <c r="B23" s="3" t="s">
+        <v>176</v>
+      </c>
+      <c r="C23" t="s">
         <v>24</v>
       </c>
-      <c r="D21" t="s">
+      <c r="D23" t="s">
         <v>24</v>
       </c>
-      <c r="E21">
+      <c r="E23">
         <v>15</v>
       </c>
-      <c r="F21" s="3" t="s">
-        <v>178</v>
-      </c>
-      <c r="G21" s="13" t="s">
+      <c r="F23" s="3" t="s">
+        <v>177</v>
+      </c>
+      <c r="G23" s="13" t="s">
+        <v>183</v>
+      </c>
+      <c r="H23" s="3" t="s">
+        <v>172</v>
+      </c>
+      <c r="I23" s="3" t="s">
+        <v>173</v>
+      </c>
+      <c r="J23" s="3" t="s">
+        <v>172</v>
+      </c>
+      <c r="K23" s="3" t="s">
+        <v>173</v>
+      </c>
+    </row>
+    <row r="24" spans="1:11" ht="255" x14ac:dyDescent="0.2">
+      <c r="A24" t="b">
+        <v>0</v>
+      </c>
+      <c r="B24" s="3" t="s">
         <v>176</v>
       </c>
-      <c r="H21" s="3" t="s">
-        <v>172</v>
-      </c>
-      <c r="I21" s="3" t="s">
-        <v>173</v>
-      </c>
-      <c r="J21" s="3" t="s">
-        <v>172</v>
-      </c>
-      <c r="K21" s="3" t="s">
-        <v>173</v>
-      </c>
-    </row>
-    <row r="22" spans="1:11" ht="17" x14ac:dyDescent="0.2">
-      <c r="A22" t="b">
-        <v>0</v>
-      </c>
-      <c r="B22" s="3" t="s">
+      <c r="C24" t="s">
+        <v>25</v>
+      </c>
+      <c r="D24" t="s">
+        <v>25</v>
+      </c>
+      <c r="E24">
+        <v>16</v>
+      </c>
+      <c r="F24" s="3" t="s">
         <v>177</v>
       </c>
-      <c r="C22" t="s">
-        <v>25</v>
-      </c>
-      <c r="D22" t="s">
-        <v>25</v>
-      </c>
-      <c r="E22">
-        <v>16</v>
-      </c>
-      <c r="F22" s="3" t="s">
-        <v>178</v>
-      </c>
-      <c r="G22" s="13" t="s">
+      <c r="G24" s="13" t="s">
+        <v>183</v>
+      </c>
+      <c r="H24" s="3" t="s">
+        <v>172</v>
+      </c>
+      <c r="I24" s="3" t="s">
+        <v>173</v>
+      </c>
+      <c r="J24" s="3" t="s">
+        <v>172</v>
+      </c>
+      <c r="K24" s="3" t="s">
+        <v>173</v>
+      </c>
+    </row>
+    <row r="25" spans="1:11" ht="255" x14ac:dyDescent="0.2">
+      <c r="A25" t="b">
+        <v>0</v>
+      </c>
+      <c r="B25" s="3" t="s">
         <v>176</v>
       </c>
-      <c r="H22" s="3" t="s">
-        <v>172</v>
-      </c>
-      <c r="I22" s="3" t="s">
-        <v>173</v>
-      </c>
-      <c r="J22" s="3" t="s">
-        <v>172</v>
-      </c>
-      <c r="K22" s="3" t="s">
-        <v>173</v>
-      </c>
-    </row>
-    <row r="23" spans="1:11" ht="17" x14ac:dyDescent="0.2">
-      <c r="A23" t="b">
-        <v>0</v>
-      </c>
-      <c r="B23" s="3" t="s">
+      <c r="C25" s="3" t="s">
+        <v>37</v>
+      </c>
+      <c r="D25" s="3" t="s">
+        <v>37</v>
+      </c>
+      <c r="E25">
+        <v>29</v>
+      </c>
+      <c r="F25" s="3" t="s">
         <v>177</v>
       </c>
-      <c r="C23" t="s">
+      <c r="G25" s="13" t="s">
+        <v>183</v>
+      </c>
+      <c r="H25" s="3" t="s">
+        <v>172</v>
+      </c>
+      <c r="I25" s="3" t="s">
+        <v>173</v>
+      </c>
+      <c r="J25" s="3" t="s">
+        <v>172</v>
+      </c>
+      <c r="K25" s="3" t="s">
+        <v>173</v>
+      </c>
+    </row>
+    <row r="26" spans="1:11" ht="255" x14ac:dyDescent="0.2">
+      <c r="A26" t="b">
+        <v>0</v>
+      </c>
+      <c r="B26" s="3" t="s">
+        <v>176</v>
+      </c>
+      <c r="C26" t="s">
+        <v>38</v>
+      </c>
+      <c r="D26" t="s">
+        <v>38</v>
+      </c>
+      <c r="E26">
+        <v>30</v>
+      </c>
+      <c r="F26" s="3" t="s">
+        <v>177</v>
+      </c>
+      <c r="G26" s="13" t="s">
+        <v>183</v>
+      </c>
+      <c r="H26" s="3" t="s">
+        <v>172</v>
+      </c>
+      <c r="I26" s="3" t="s">
+        <v>173</v>
+      </c>
+      <c r="J26" s="3" t="s">
+        <v>172</v>
+      </c>
+      <c r="K26" s="3" t="s">
+        <v>173</v>
+      </c>
+    </row>
+    <row r="27" spans="1:11" ht="272" x14ac:dyDescent="0.2">
+      <c r="A27" t="b">
+        <v>0</v>
+      </c>
+      <c r="B27" s="3" t="s">
+        <v>176</v>
+      </c>
+      <c r="C27" t="s">
+        <v>42</v>
+      </c>
+      <c r="D27" t="s">
+        <v>42</v>
+      </c>
+      <c r="E27">
+        <v>34</v>
+      </c>
+      <c r="F27" s="3" t="s">
+        <v>177</v>
+      </c>
+      <c r="G27" s="13" t="s">
+        <v>182</v>
+      </c>
+      <c r="H27" s="3" t="s">
+        <v>172</v>
+      </c>
+      <c r="I27" s="3" t="s">
+        <v>173</v>
+      </c>
+      <c r="J27" s="3" t="s">
+        <v>172</v>
+      </c>
+      <c r="K27" s="3" t="s">
+        <v>173</v>
+      </c>
+    </row>
+    <row r="28" spans="1:11" ht="255" x14ac:dyDescent="0.2">
+      <c r="A28" t="b">
+        <v>0</v>
+      </c>
+      <c r="B28" s="3" t="s">
+        <v>176</v>
+      </c>
+      <c r="C28" t="s">
         <v>26</v>
       </c>
-      <c r="D23" t="s">
+      <c r="D28" t="s">
         <v>26</v>
       </c>
-      <c r="E23">
+      <c r="E28">
         <v>17</v>
       </c>
-      <c r="F23" s="3" t="s">
-        <v>178</v>
-      </c>
-      <c r="G23" s="13" t="s">
+      <c r="F28" s="3" t="s">
+        <v>177</v>
+      </c>
+      <c r="G28" s="13" t="s">
+        <v>183</v>
+      </c>
+      <c r="H28" s="3" t="s">
+        <v>172</v>
+      </c>
+      <c r="I28" s="3" t="s">
+        <v>173</v>
+      </c>
+      <c r="J28" s="3" t="s">
+        <v>172</v>
+      </c>
+      <c r="K28" s="3" t="s">
+        <v>173</v>
+      </c>
+    </row>
+    <row r="29" spans="1:11" ht="306" x14ac:dyDescent="0.2">
+      <c r="A29" t="b">
+        <v>0</v>
+      </c>
+      <c r="B29" s="3" t="s">
         <v>176</v>
       </c>
-      <c r="H23" s="3" t="s">
-        <v>172</v>
-      </c>
-      <c r="I23" s="3" t="s">
-        <v>173</v>
-      </c>
-      <c r="J23" s="3" t="s">
-        <v>172</v>
-      </c>
-      <c r="K23" s="3" t="s">
-        <v>173</v>
-      </c>
-    </row>
-    <row r="24" spans="1:11" ht="17" x14ac:dyDescent="0.2">
-      <c r="A24" t="b">
-        <v>0</v>
-      </c>
-      <c r="B24" s="3" t="s">
+      <c r="C29" t="s">
+        <v>40</v>
+      </c>
+      <c r="D29" t="s">
+        <v>40</v>
+      </c>
+      <c r="E29">
+        <v>32</v>
+      </c>
+      <c r="F29" s="3" t="s">
         <v>177</v>
       </c>
-      <c r="C24" t="s">
+      <c r="G29" s="13" t="s">
+        <v>179</v>
+      </c>
+      <c r="H29" s="3" t="s">
+        <v>172</v>
+      </c>
+      <c r="I29" s="3" t="s">
+        <v>173</v>
+      </c>
+      <c r="J29" s="3" t="s">
+        <v>172</v>
+      </c>
+      <c r="K29" s="3" t="s">
+        <v>173</v>
+      </c>
+    </row>
+    <row r="30" spans="1:11" ht="255" x14ac:dyDescent="0.2">
+      <c r="A30" t="b">
+        <v>0</v>
+      </c>
+      <c r="B30" s="3" t="s">
+        <v>176</v>
+      </c>
+      <c r="C30" t="s">
         <v>27</v>
       </c>
-      <c r="D24" t="s">
+      <c r="D30" t="s">
         <v>27</v>
       </c>
-      <c r="E24">
+      <c r="E30">
         <v>18</v>
       </c>
-      <c r="F24" s="3" t="s">
-        <v>178</v>
-      </c>
-      <c r="G24" s="13" t="s">
+      <c r="F30" s="3" t="s">
+        <v>177</v>
+      </c>
+      <c r="G30" s="13" t="s">
+        <v>183</v>
+      </c>
+      <c r="H30" s="3" t="s">
+        <v>172</v>
+      </c>
+      <c r="I30" s="3" t="s">
+        <v>173</v>
+      </c>
+      <c r="J30" s="3" t="s">
+        <v>172</v>
+      </c>
+      <c r="K30" s="3" t="s">
+        <v>173</v>
+      </c>
+    </row>
+    <row r="31" spans="1:11" ht="255" x14ac:dyDescent="0.2">
+      <c r="A31" t="b">
+        <v>0</v>
+      </c>
+      <c r="B31" s="3" t="s">
         <v>176</v>
       </c>
-      <c r="H24" s="3" t="s">
-        <v>172</v>
-      </c>
-      <c r="I24" s="3" t="s">
-        <v>173</v>
-      </c>
-      <c r="J24" s="3" t="s">
-        <v>172</v>
-      </c>
-      <c r="K24" s="3" t="s">
-        <v>173</v>
-      </c>
-    </row>
-    <row r="25" spans="1:11" ht="17" x14ac:dyDescent="0.2">
-      <c r="A25" t="b">
-        <v>0</v>
-      </c>
-      <c r="B25" s="3" t="s">
+      <c r="C31" t="s">
+        <v>28</v>
+      </c>
+      <c r="D31" t="s">
+        <v>28</v>
+      </c>
+      <c r="E31">
+        <v>19</v>
+      </c>
+      <c r="F31" s="3" t="s">
         <v>177</v>
       </c>
-      <c r="C25" t="s">
-        <v>28</v>
-      </c>
-      <c r="D25" t="s">
-        <v>28</v>
-      </c>
-      <c r="E25">
-        <v>19</v>
-      </c>
-      <c r="F25" s="3" t="s">
-        <v>178</v>
-      </c>
-      <c r="G25" s="13" t="s">
+      <c r="G31" s="13" t="s">
+        <v>183</v>
+      </c>
+      <c r="H31" s="3" t="s">
+        <v>172</v>
+      </c>
+      <c r="I31" s="3" t="s">
+        <v>173</v>
+      </c>
+      <c r="J31" s="3" t="s">
+        <v>172</v>
+      </c>
+      <c r="K31" s="3" t="s">
+        <v>173</v>
+      </c>
+    </row>
+    <row r="32" spans="1:11" ht="255" x14ac:dyDescent="0.2">
+      <c r="A32" t="b">
+        <v>0</v>
+      </c>
+      <c r="B32" s="3" t="s">
         <v>176</v>
       </c>
-      <c r="H25" s="3" t="s">
-        <v>172</v>
-      </c>
-      <c r="I25" s="3" t="s">
-        <v>173</v>
-      </c>
-      <c r="J25" s="3" t="s">
-        <v>172</v>
-      </c>
-      <c r="K25" s="3" t="s">
-        <v>173</v>
-      </c>
-    </row>
-    <row r="26" spans="1:11" ht="17" x14ac:dyDescent="0.2">
-      <c r="A26" t="b">
-        <v>0</v>
-      </c>
-      <c r="B26" s="3" t="s">
+      <c r="C32" t="s">
+        <v>29</v>
+      </c>
+      <c r="D32" t="s">
+        <v>29</v>
+      </c>
+      <c r="E32">
+        <v>20</v>
+      </c>
+      <c r="F32" s="3" t="s">
         <v>177</v>
       </c>
-      <c r="C26" t="s">
-        <v>29</v>
-      </c>
-      <c r="D26" t="s">
-        <v>29</v>
-      </c>
-      <c r="E26">
-        <v>20</v>
-      </c>
-      <c r="F26" s="3" t="s">
-        <v>178</v>
-      </c>
-      <c r="G26" s="13" t="s">
+      <c r="G32" s="13" t="s">
+        <v>183</v>
+      </c>
+      <c r="H32" s="3" t="s">
+        <v>172</v>
+      </c>
+      <c r="I32" s="3" t="s">
+        <v>173</v>
+      </c>
+      <c r="J32" s="3" t="s">
+        <v>172</v>
+      </c>
+      <c r="K32" s="3" t="s">
+        <v>173</v>
+      </c>
+    </row>
+    <row r="33" spans="1:11" ht="272" x14ac:dyDescent="0.2">
+      <c r="A33" t="b">
+        <v>0</v>
+      </c>
+      <c r="B33" s="3" t="s">
         <v>176</v>
       </c>
-      <c r="H26" s="3" t="s">
-        <v>172</v>
-      </c>
-      <c r="I26" s="3" t="s">
-        <v>173</v>
-      </c>
-      <c r="J26" s="3" t="s">
-        <v>172</v>
-      </c>
-      <c r="K26" s="3" t="s">
-        <v>173</v>
-      </c>
-    </row>
-    <row r="27" spans="1:11" ht="17" x14ac:dyDescent="0.2">
-      <c r="A27" t="b">
-        <v>0</v>
-      </c>
-      <c r="B27" s="3" t="s">
+      <c r="C33" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="D33" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="E33">
+        <v>21</v>
+      </c>
+      <c r="F33" s="3" t="s">
         <v>177</v>
       </c>
-      <c r="C27" t="s">
-        <v>31</v>
-      </c>
-      <c r="D27" t="s">
-        <v>31</v>
-      </c>
-      <c r="E27">
-        <v>23</v>
-      </c>
-      <c r="F27" s="3" t="s">
-        <v>178</v>
-      </c>
-      <c r="G27" s="13" t="s">
+      <c r="G33" s="13" t="s">
+        <v>182</v>
+      </c>
+      <c r="H33" s="3" t="s">
+        <v>172</v>
+      </c>
+      <c r="I33" s="3" t="s">
+        <v>173</v>
+      </c>
+      <c r="J33" s="3" t="s">
+        <v>172</v>
+      </c>
+      <c r="K33" s="3" t="s">
+        <v>173</v>
+      </c>
+    </row>
+    <row r="34" spans="1:11" ht="255" x14ac:dyDescent="0.2">
+      <c r="A34" t="b">
+        <v>0</v>
+      </c>
+      <c r="B34" s="3" t="s">
         <v>176</v>
       </c>
-      <c r="H27" s="3" t="s">
-        <v>172</v>
-      </c>
-      <c r="I27" s="3" t="s">
-        <v>173</v>
-      </c>
-      <c r="J27" s="3" t="s">
-        <v>172</v>
-      </c>
-      <c r="K27" s="3" t="s">
-        <v>173</v>
-      </c>
-    </row>
-    <row r="28" spans="1:11" ht="17" x14ac:dyDescent="0.2">
-      <c r="A28" t="b">
-        <v>0</v>
-      </c>
-      <c r="B28" s="3" t="s">
+      <c r="C34" t="s">
+        <v>51</v>
+      </c>
+      <c r="D34" t="s">
+        <v>51</v>
+      </c>
+      <c r="E34">
+        <v>43</v>
+      </c>
+      <c r="F34" s="3" t="s">
         <v>177</v>
       </c>
-      <c r="C28" t="s">
-        <v>32</v>
-      </c>
-      <c r="D28" t="s">
-        <v>32</v>
-      </c>
-      <c r="E28">
-        <v>24</v>
-      </c>
-      <c r="F28" s="3" t="s">
-        <v>178</v>
-      </c>
-      <c r="G28" s="13" t="s">
+      <c r="G34" s="13" t="s">
+        <v>183</v>
+      </c>
+      <c r="H34" s="3" t="s">
+        <v>172</v>
+      </c>
+      <c r="I34" s="3" t="s">
+        <v>173</v>
+      </c>
+      <c r="J34" s="3" t="s">
+        <v>172</v>
+      </c>
+      <c r="K34" s="3" t="s">
+        <v>173</v>
+      </c>
+    </row>
+    <row r="35" spans="1:11" ht="356" x14ac:dyDescent="0.2">
+      <c r="A35" t="b">
+        <v>0</v>
+      </c>
+      <c r="B35" s="3" t="s">
         <v>176</v>
       </c>
-      <c r="H28" s="3" t="s">
-        <v>172</v>
-      </c>
-      <c r="I28" s="3" t="s">
-        <v>173</v>
-      </c>
-      <c r="J28" s="3" t="s">
-        <v>172</v>
-      </c>
-      <c r="K28" s="3" t="s">
-        <v>173</v>
-      </c>
-    </row>
-    <row r="29" spans="1:11" ht="17" x14ac:dyDescent="0.2">
-      <c r="A29" t="b">
-        <v>0</v>
-      </c>
-      <c r="B29" s="3" t="s">
+      <c r="C35" s="3" t="s">
+        <v>30</v>
+      </c>
+      <c r="D35" s="3" t="s">
+        <v>30</v>
+      </c>
+      <c r="E35">
+        <v>22</v>
+      </c>
+      <c r="F35" s="3" t="s">
         <v>177</v>
       </c>
-      <c r="C29" t="s">
-        <v>33</v>
-      </c>
-      <c r="D29" t="s">
-        <v>33</v>
-      </c>
-      <c r="E29">
-        <v>25</v>
-      </c>
-      <c r="F29" s="3" t="s">
-        <v>178</v>
-      </c>
-      <c r="G29" s="13" t="s">
-        <v>176</v>
-      </c>
-      <c r="H29" s="3" t="s">
-        <v>172</v>
-      </c>
-      <c r="I29" s="3" t="s">
-        <v>173</v>
-      </c>
-      <c r="J29" s="3" t="s">
-        <v>172</v>
-      </c>
-      <c r="K29" s="3" t="s">
-        <v>173</v>
-      </c>
-    </row>
-    <row r="30" spans="1:11" ht="17" x14ac:dyDescent="0.2">
-      <c r="A30" t="b">
-        <v>0</v>
-      </c>
-      <c r="B30" s="3" t="s">
-        <v>177</v>
-      </c>
-      <c r="C30" t="s">
-        <v>34</v>
-      </c>
-      <c r="D30" t="s">
-        <v>34</v>
-      </c>
-      <c r="E30">
-        <v>26</v>
-      </c>
-      <c r="F30" s="3" t="s">
-        <v>178</v>
-      </c>
-      <c r="G30" s="13" t="s">
-        <v>176</v>
-      </c>
-      <c r="H30" s="3" t="s">
-        <v>172</v>
-      </c>
-      <c r="I30" s="3" t="s">
-        <v>173</v>
-      </c>
-      <c r="J30" s="3" t="s">
-        <v>172</v>
-      </c>
-      <c r="K30" s="3" t="s">
-        <v>173</v>
-      </c>
-    </row>
-    <row r="31" spans="1:11" ht="17" x14ac:dyDescent="0.2">
-      <c r="A31" t="b">
-        <v>0</v>
-      </c>
-      <c r="B31" s="3" t="s">
-        <v>177</v>
-      </c>
-      <c r="C31" t="s">
-        <v>36</v>
-      </c>
-      <c r="D31" t="s">
-        <v>36</v>
-      </c>
-      <c r="E31">
-        <v>28</v>
-      </c>
-      <c r="F31" s="3" t="s">
-        <v>178</v>
-      </c>
-      <c r="G31" s="13" t="s">
-        <v>176</v>
-      </c>
-      <c r="H31" s="3" t="s">
-        <v>172</v>
-      </c>
-      <c r="I31" s="3" t="s">
-        <v>173</v>
-      </c>
-      <c r="J31" s="3" t="s">
-        <v>172</v>
-      </c>
-      <c r="K31" s="3" t="s">
-        <v>173</v>
-      </c>
-    </row>
-    <row r="32" spans="1:11" ht="17" x14ac:dyDescent="0.2">
-      <c r="A32" t="b">
-        <v>0</v>
-      </c>
-      <c r="B32" s="3" t="s">
-        <v>177</v>
-      </c>
-      <c r="C32" t="s">
-        <v>38</v>
-      </c>
-      <c r="D32" t="s">
-        <v>38</v>
-      </c>
-      <c r="E32">
-        <v>30</v>
-      </c>
-      <c r="F32" s="3" t="s">
-        <v>178</v>
-      </c>
-      <c r="G32" s="13" t="s">
-        <v>176</v>
-      </c>
-      <c r="H32" s="3" t="s">
-        <v>172</v>
-      </c>
-      <c r="I32" s="3" t="s">
-        <v>173</v>
-      </c>
-      <c r="J32" s="3" t="s">
-        <v>172</v>
-      </c>
-      <c r="K32" s="3" t="s">
-        <v>173</v>
-      </c>
-    </row>
-    <row r="33" spans="1:11" ht="119" x14ac:dyDescent="0.2">
-      <c r="A33" t="b">
-        <v>0</v>
-      </c>
-      <c r="B33" s="3" t="s">
-        <v>177</v>
-      </c>
-      <c r="C33" t="s">
-        <v>40</v>
-      </c>
-      <c r="D33" t="s">
-        <v>40</v>
-      </c>
-      <c r="E33">
-        <v>32</v>
-      </c>
-      <c r="F33" s="3" t="s">
-        <v>178</v>
-      </c>
-      <c r="G33" s="13" t="s">
-        <v>180</v>
-      </c>
-      <c r="H33" s="3" t="s">
-        <v>172</v>
-      </c>
-      <c r="I33" s="3" t="s">
-        <v>173</v>
-      </c>
-      <c r="J33" s="3" t="s">
-        <v>172</v>
-      </c>
-      <c r="K33" s="3" t="s">
-        <v>173</v>
-      </c>
-    </row>
-    <row r="34" spans="1:11" ht="17" x14ac:dyDescent="0.2">
-      <c r="A34" t="b">
-        <v>0</v>
-      </c>
-      <c r="B34" s="3" t="s">
-        <v>177</v>
-      </c>
-      <c r="C34" t="s">
-        <v>41</v>
-      </c>
-      <c r="D34" t="s">
-        <v>41</v>
-      </c>
-      <c r="E34">
-        <v>33</v>
-      </c>
-      <c r="F34" s="3" t="s">
-        <v>178</v>
-      </c>
-      <c r="G34" s="13" t="s">
-        <v>176</v>
-      </c>
-      <c r="H34" s="3" t="s">
-        <v>172</v>
-      </c>
-      <c r="I34" s="3" t="s">
-        <v>173</v>
-      </c>
-      <c r="J34" s="3" t="s">
-        <v>172</v>
-      </c>
-      <c r="K34" s="3" t="s">
-        <v>173</v>
-      </c>
-    </row>
-    <row r="35" spans="1:11" ht="17" x14ac:dyDescent="0.2">
-      <c r="A35" t="b">
-        <v>0</v>
-      </c>
-      <c r="B35" s="3" t="s">
-        <v>177</v>
-      </c>
-      <c r="C35" t="s">
-        <v>42</v>
-      </c>
-      <c r="D35" t="s">
-        <v>42</v>
-      </c>
-      <c r="E35">
-        <v>34</v>
-      </c>
-      <c r="F35" s="3" t="s">
-        <v>178</v>
-      </c>
       <c r="G35" s="13" t="s">
-        <v>176</v>
+        <v>181</v>
       </c>
       <c r="H35" s="3" t="s">
         <v>172</v>
@@ -3207,343 +3219,346 @@
     </row>
     <row r="36" spans="1:11" ht="17" x14ac:dyDescent="0.2">
       <c r="A36" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="B36" s="3" t="s">
+        <v>176</v>
+      </c>
+      <c r="C36" t="s">
+        <v>53</v>
+      </c>
+      <c r="D36" t="s">
+        <v>53</v>
+      </c>
+      <c r="E36">
+        <v>45</v>
+      </c>
+      <c r="F36" s="3" t="s">
         <v>177</v>
       </c>
-      <c r="C36" t="s">
-        <v>43</v>
-      </c>
-      <c r="D36" t="s">
-        <v>43</v>
-      </c>
-      <c r="E36">
-        <v>35</v>
-      </c>
-      <c r="F36" s="3" t="s">
+      <c r="G36" s="12" t="s">
         <v>178</v>
       </c>
-      <c r="G36" s="13" t="s">
+      <c r="H36" s="3" t="s">
+        <v>172</v>
+      </c>
+      <c r="I36" s="3" t="s">
+        <v>173</v>
+      </c>
+      <c r="J36" s="3" t="s">
+        <v>172</v>
+      </c>
+      <c r="K36" s="3" t="s">
+        <v>173</v>
+      </c>
+    </row>
+    <row r="37" spans="1:11" ht="255" x14ac:dyDescent="0.2">
+      <c r="A37" t="b">
+        <v>0</v>
+      </c>
+      <c r="B37" s="3" t="s">
         <v>176</v>
       </c>
-      <c r="H36" s="3" t="s">
-        <v>172</v>
-      </c>
-      <c r="I36" s="3" t="s">
-        <v>173</v>
-      </c>
-      <c r="J36" s="3" t="s">
-        <v>172</v>
-      </c>
-      <c r="K36" s="3" t="s">
-        <v>173</v>
-      </c>
-    </row>
-    <row r="37" spans="1:11" ht="17" x14ac:dyDescent="0.2">
-      <c r="A37" t="b">
-        <v>0</v>
-      </c>
-      <c r="B37" s="3" t="s">
+      <c r="C37" t="s">
+        <v>45</v>
+      </c>
+      <c r="D37" t="s">
+        <v>45</v>
+      </c>
+      <c r="E37">
+        <v>37</v>
+      </c>
+      <c r="F37" s="3" t="s">
         <v>177</v>
       </c>
-      <c r="C37" t="s">
+      <c r="G37" s="13" t="s">
+        <v>183</v>
+      </c>
+      <c r="H37" s="3" t="s">
+        <v>172</v>
+      </c>
+      <c r="I37" s="3" t="s">
+        <v>173</v>
+      </c>
+      <c r="J37" s="3" t="s">
+        <v>172</v>
+      </c>
+      <c r="K37" s="3" t="s">
+        <v>173</v>
+      </c>
+    </row>
+    <row r="38" spans="1:11" ht="255" x14ac:dyDescent="0.2">
+      <c r="A38" t="b">
+        <v>0</v>
+      </c>
+      <c r="B38" s="3" t="s">
+        <v>176</v>
+      </c>
+      <c r="C38" s="3" t="s">
+        <v>39</v>
+      </c>
+      <c r="D38" s="3" t="s">
+        <v>39</v>
+      </c>
+      <c r="E38">
+        <v>31</v>
+      </c>
+      <c r="F38" s="3" t="s">
+        <v>177</v>
+      </c>
+      <c r="G38" s="13" t="s">
+        <v>183</v>
+      </c>
+      <c r="H38" s="3" t="s">
+        <v>172</v>
+      </c>
+      <c r="I38" s="3" t="s">
+        <v>173</v>
+      </c>
+      <c r="J38" s="3" t="s">
+        <v>172</v>
+      </c>
+      <c r="K38" s="3" t="s">
+        <v>173</v>
+      </c>
+    </row>
+    <row r="39" spans="1:11" ht="255" x14ac:dyDescent="0.2">
+      <c r="A39" t="b">
+        <v>0</v>
+      </c>
+      <c r="B39" s="3" t="s">
+        <v>176</v>
+      </c>
+      <c r="C39" t="s">
+        <v>31</v>
+      </c>
+      <c r="D39" t="s">
+        <v>31</v>
+      </c>
+      <c r="E39">
+        <v>23</v>
+      </c>
+      <c r="F39" s="3" t="s">
+        <v>177</v>
+      </c>
+      <c r="G39" s="13" t="s">
+        <v>183</v>
+      </c>
+      <c r="H39" s="3" t="s">
+        <v>172</v>
+      </c>
+      <c r="I39" s="3" t="s">
+        <v>173</v>
+      </c>
+      <c r="J39" s="3" t="s">
+        <v>172</v>
+      </c>
+      <c r="K39" s="3" t="s">
+        <v>173</v>
+      </c>
+    </row>
+    <row r="40" spans="1:11" ht="255" x14ac:dyDescent="0.2">
+      <c r="A40" t="b">
+        <v>0</v>
+      </c>
+      <c r="B40" s="3" t="s">
+        <v>176</v>
+      </c>
+      <c r="C40" t="s">
+        <v>32</v>
+      </c>
+      <c r="D40" t="s">
+        <v>32</v>
+      </c>
+      <c r="E40">
+        <v>24</v>
+      </c>
+      <c r="F40" s="3" t="s">
+        <v>177</v>
+      </c>
+      <c r="G40" s="13" t="s">
+        <v>183</v>
+      </c>
+      <c r="H40" s="3" t="s">
+        <v>172</v>
+      </c>
+      <c r="I40" s="3" t="s">
+        <v>173</v>
+      </c>
+      <c r="J40" s="3" t="s">
+        <v>172</v>
+      </c>
+      <c r="K40" s="3" t="s">
+        <v>173</v>
+      </c>
+    </row>
+    <row r="41" spans="1:11" ht="255" x14ac:dyDescent="0.2">
+      <c r="A41" t="b">
+        <v>0</v>
+      </c>
+      <c r="B41" s="3" t="s">
+        <v>176</v>
+      </c>
+      <c r="C41" t="s">
+        <v>33</v>
+      </c>
+      <c r="D41" t="s">
+        <v>33</v>
+      </c>
+      <c r="E41">
+        <v>25</v>
+      </c>
+      <c r="F41" s="3" t="s">
+        <v>177</v>
+      </c>
+      <c r="G41" s="13" t="s">
+        <v>183</v>
+      </c>
+      <c r="H41" s="3" t="s">
+        <v>172</v>
+      </c>
+      <c r="I41" s="3" t="s">
+        <v>173</v>
+      </c>
+      <c r="J41" s="3" t="s">
+        <v>172</v>
+      </c>
+      <c r="K41" s="3" t="s">
+        <v>173</v>
+      </c>
+    </row>
+    <row r="42" spans="1:11" ht="255" x14ac:dyDescent="0.2">
+      <c r="A42" t="b">
+        <v>0</v>
+      </c>
+      <c r="B42" s="3" t="s">
+        <v>176</v>
+      </c>
+      <c r="C42" t="s">
+        <v>52</v>
+      </c>
+      <c r="D42" t="s">
+        <v>52</v>
+      </c>
+      <c r="E42">
         <v>44</v>
       </c>
-      <c r="D37" t="s">
-        <v>44</v>
-      </c>
-      <c r="E37">
-        <v>36</v>
-      </c>
-      <c r="F37" s="3" t="s">
-        <v>178</v>
-      </c>
-      <c r="G37" s="13" t="s">
+      <c r="F42" s="3" t="s">
+        <v>177</v>
+      </c>
+      <c r="G42" s="13" t="s">
+        <v>183</v>
+      </c>
+      <c r="H42" s="3" t="s">
+        <v>172</v>
+      </c>
+      <c r="I42" s="3" t="s">
+        <v>173</v>
+      </c>
+      <c r="J42" s="3" t="s">
+        <v>172</v>
+      </c>
+      <c r="K42" s="3" t="s">
+        <v>173</v>
+      </c>
+    </row>
+    <row r="43" spans="1:11" ht="255" x14ac:dyDescent="0.2">
+      <c r="A43" t="b">
+        <v>0</v>
+      </c>
+      <c r="B43" s="3" t="s">
         <v>176</v>
       </c>
-      <c r="H37" s="3" t="s">
-        <v>172</v>
-      </c>
-      <c r="I37" s="3" t="s">
-        <v>173</v>
-      </c>
-      <c r="J37" s="3" t="s">
-        <v>172</v>
-      </c>
-      <c r="K37" s="3" t="s">
-        <v>173</v>
-      </c>
-    </row>
-    <row r="38" spans="1:11" ht="17" x14ac:dyDescent="0.2">
-      <c r="A38" t="b">
-        <v>0</v>
-      </c>
-      <c r="B38" s="3" t="s">
+      <c r="C43" t="s">
+        <v>46</v>
+      </c>
+      <c r="D43" t="s">
+        <v>46</v>
+      </c>
+      <c r="E43">
+        <v>38</v>
+      </c>
+      <c r="F43" s="3" t="s">
         <v>177</v>
       </c>
-      <c r="C38" t="s">
-        <v>45</v>
-      </c>
-      <c r="D38" t="s">
-        <v>45</v>
-      </c>
-      <c r="E38">
-        <v>37</v>
-      </c>
-      <c r="F38" s="3" t="s">
-        <v>178</v>
-      </c>
-      <c r="G38" s="13" t="s">
+      <c r="G43" s="13" t="s">
+        <v>183</v>
+      </c>
+      <c r="H43" s="3" t="s">
+        <v>172</v>
+      </c>
+      <c r="I43" s="3" t="s">
+        <v>173</v>
+      </c>
+      <c r="J43" s="3" t="s">
+        <v>172</v>
+      </c>
+      <c r="K43" s="3" t="s">
+        <v>173</v>
+      </c>
+    </row>
+    <row r="44" spans="1:11" ht="255" x14ac:dyDescent="0.2">
+      <c r="A44" t="b">
+        <v>0</v>
+      </c>
+      <c r="B44" s="3" t="s">
         <v>176</v>
       </c>
-      <c r="H38" s="3" t="s">
-        <v>172</v>
-      </c>
-      <c r="I38" s="3" t="s">
-        <v>173</v>
-      </c>
-      <c r="J38" s="3" t="s">
-        <v>172</v>
-      </c>
-      <c r="K38" s="3" t="s">
-        <v>173</v>
-      </c>
-    </row>
-    <row r="39" spans="1:11" ht="17" x14ac:dyDescent="0.2">
-      <c r="A39" t="b">
-        <v>0</v>
-      </c>
-      <c r="B39" s="3" t="s">
+      <c r="C44" t="s">
+        <v>34</v>
+      </c>
+      <c r="D44" t="s">
+        <v>34</v>
+      </c>
+      <c r="E44">
+        <v>26</v>
+      </c>
+      <c r="F44" s="3" t="s">
         <v>177</v>
       </c>
-      <c r="C39" t="s">
-        <v>46</v>
-      </c>
-      <c r="D39" t="s">
-        <v>46</v>
-      </c>
-      <c r="E39">
-        <v>38</v>
-      </c>
-      <c r="F39" s="3" t="s">
-        <v>178</v>
-      </c>
-      <c r="G39" s="13" t="s">
-        <v>176</v>
-      </c>
-      <c r="H39" s="3" t="s">
-        <v>172</v>
-      </c>
-      <c r="I39" s="3" t="s">
-        <v>173</v>
-      </c>
-      <c r="J39" s="3" t="s">
-        <v>172</v>
-      </c>
-      <c r="K39" s="3" t="s">
-        <v>173</v>
-      </c>
-    </row>
-    <row r="40" spans="1:11" ht="17" x14ac:dyDescent="0.2">
-      <c r="A40" t="b">
-        <v>0</v>
-      </c>
-      <c r="B40" s="3" t="s">
-        <v>177</v>
-      </c>
-      <c r="C40" t="s">
-        <v>47</v>
-      </c>
-      <c r="D40" t="s">
-        <v>47</v>
-      </c>
-      <c r="E40">
-        <v>39</v>
-      </c>
-      <c r="F40" s="3" t="s">
-        <v>178</v>
-      </c>
-      <c r="G40" s="13" t="s">
-        <v>176</v>
-      </c>
-      <c r="H40" s="3" t="s">
-        <v>172</v>
-      </c>
-      <c r="I40" s="3" t="s">
-        <v>173</v>
-      </c>
-      <c r="J40" s="3" t="s">
-        <v>172</v>
-      </c>
-      <c r="K40" s="3" t="s">
-        <v>173</v>
-      </c>
-    </row>
-    <row r="41" spans="1:11" ht="17" x14ac:dyDescent="0.2">
-      <c r="A41" t="b">
-        <v>0</v>
-      </c>
-      <c r="B41" s="3" t="s">
-        <v>177</v>
-      </c>
-      <c r="C41" t="s">
-        <v>49</v>
-      </c>
-      <c r="D41" t="s">
-        <v>49</v>
-      </c>
-      <c r="E41">
-        <v>41</v>
-      </c>
-      <c r="F41" s="3" t="s">
-        <v>178</v>
-      </c>
-      <c r="G41" s="13" t="s">
-        <v>176</v>
-      </c>
-      <c r="H41" s="3" t="s">
-        <v>172</v>
-      </c>
-      <c r="I41" s="3" t="s">
-        <v>173</v>
-      </c>
-      <c r="J41" s="3" t="s">
-        <v>172</v>
-      </c>
-      <c r="K41" s="3" t="s">
-        <v>173</v>
-      </c>
-    </row>
-    <row r="42" spans="1:11" ht="17" x14ac:dyDescent="0.2">
-      <c r="A42" t="b">
-        <v>0</v>
-      </c>
-      <c r="B42" s="3" t="s">
-        <v>177</v>
-      </c>
-      <c r="C42" t="s">
-        <v>51</v>
-      </c>
-      <c r="D42" t="s">
-        <v>51</v>
-      </c>
-      <c r="E42">
-        <v>43</v>
-      </c>
-      <c r="F42" s="3" t="s">
-        <v>178</v>
-      </c>
-      <c r="G42" s="13" t="s">
-        <v>176</v>
-      </c>
-      <c r="H42" s="3" t="s">
-        <v>172</v>
-      </c>
-      <c r="I42" s="3" t="s">
-        <v>173</v>
-      </c>
-      <c r="J42" s="3" t="s">
-        <v>172</v>
-      </c>
-      <c r="K42" s="3" t="s">
-        <v>173</v>
-      </c>
-    </row>
-    <row r="43" spans="1:11" ht="17" x14ac:dyDescent="0.2">
-      <c r="A43" t="b">
-        <v>0</v>
-      </c>
-      <c r="B43" s="3" t="s">
-        <v>177</v>
-      </c>
-      <c r="C43" t="s">
-        <v>52</v>
-      </c>
-      <c r="D43" t="s">
-        <v>52</v>
-      </c>
-      <c r="E43">
-        <v>44</v>
-      </c>
-      <c r="F43" s="3" t="s">
-        <v>178</v>
-      </c>
-      <c r="G43" s="13" t="s">
-        <v>176</v>
-      </c>
-      <c r="H43" s="3" t="s">
-        <v>172</v>
-      </c>
-      <c r="I43" s="3" t="s">
-        <v>173</v>
-      </c>
-      <c r="J43" s="3" t="s">
-        <v>172</v>
-      </c>
-      <c r="K43" s="3" t="s">
-        <v>173</v>
-      </c>
-    </row>
-    <row r="44" spans="1:11" ht="17" x14ac:dyDescent="0.2">
-      <c r="A44" t="b">
+      <c r="G44" s="13" t="s">
+        <v>183</v>
+      </c>
+      <c r="H44" s="3" t="s">
+        <v>172</v>
+      </c>
+      <c r="I44" s="3" t="s">
+        <v>173</v>
+      </c>
+      <c r="J44" s="3" t="s">
+        <v>172</v>
+      </c>
+      <c r="K44" s="3" t="s">
+        <v>173</v>
+      </c>
+    </row>
+    <row r="51" spans="3:4" x14ac:dyDescent="0.2">
+      <c r="C51" s="11" t="s">
+        <v>175</v>
+      </c>
+      <c r="D51" s="11"/>
+    </row>
+    <row r="52" spans="3:4" x14ac:dyDescent="0.2">
+      <c r="C52" s="14">
         <v>1</v>
       </c>
-      <c r="B44" s="3" t="s">
-        <v>177</v>
-      </c>
-      <c r="C44" t="s">
-        <v>53</v>
-      </c>
-      <c r="D44" t="s">
-        <v>53</v>
-      </c>
-      <c r="E44">
-        <v>45</v>
-      </c>
-      <c r="F44" s="3" t="s">
-        <v>178</v>
-      </c>
-      <c r="G44" s="12" t="s">
-        <v>179</v>
-      </c>
-      <c r="H44" s="3" t="s">
-        <v>172</v>
-      </c>
-      <c r="I44" s="3" t="s">
-        <v>173</v>
-      </c>
-      <c r="J44" s="3" t="s">
-        <v>172</v>
-      </c>
-      <c r="K44" s="3" t="s">
-        <v>173</v>
-      </c>
-    </row>
-    <row r="45" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="C45" s="11" t="s">
-        <v>175</v>
-      </c>
-      <c r="D45" s="11"/>
-    </row>
-    <row r="46" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="C46" s="14">
-        <v>1</v>
-      </c>
-      <c r="D46" s="11" t="s">
+      <c r="D52" s="11" t="s">
         <v>174</v>
       </c>
     </row>
-    <row r="47" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="C47" s="14">
+    <row r="53" spans="3:4" x14ac:dyDescent="0.2">
+      <c r="C53" s="14">
         <v>40</v>
       </c>
-      <c r="D47" s="11" t="s">
+      <c r="D53" s="11" t="s">
         <v>48</v>
       </c>
     </row>
   </sheetData>
   <autoFilter ref="A1:K47" xr:uid="{A63BE434-9ED0-E94E-BE21-7A21279D6729}"/>
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:K44">
+    <sortCondition ref="C44"/>
+  </sortState>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>

</xml_diff>